<commit_message>
feat: add backend database clinic deduplication endpoint
</commit_message>
<xml_diff>
--- a/dentai-web/selenium-tests/test-report.xlsx
+++ b/dentai-web/selenium-tests/test-report.xlsx
@@ -427,7 +427,7 @@
         <v>Error Details</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
         <v>DentAI Complete End-to-End Application Testing</v>
       </c>
@@ -435,17 +435,16 @@
         <v>1. Should register a new Dentist and create a Clinic profile</v>
       </c>
       <c r="C2" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="D2">
-        <v>39588</v>
+        <v>11636</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-07-09T19:15:41.438Z</v>
-      </c>
-      <c r="F2" t="str" xml:space="preserve">
-        <v xml:space="preserve">Logout did not redirect to /login within 15s
-Wait timed out after 15093ms</v>
+        <v>2026-07-11T04:11:52.582Z</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -459,16 +458,16 @@
         <v>PASS</v>
       </c>
       <c r="D3">
-        <v>14450</v>
+        <v>7574</v>
       </c>
       <c r="E3" t="str">
-        <v>2026-07-09T19:15:57.754Z</v>
+        <v>2026-07-11T04:12:00.158Z</v>
       </c>
       <c r="F3" t="str">
         <v/>
       </c>
     </row>
-    <row r="4" xml:space="preserve">
+    <row r="4">
       <c r="A4" t="str">
         <v>DentAI Complete End-to-End Application Testing</v>
       </c>
@@ -476,20 +475,19 @@
         <v>3. Should complete the Symptom Checker Diagnostic Wizard</v>
       </c>
       <c r="C4" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="D4">
-        <v>11252</v>
+        <v>2457</v>
       </c>
       <c r="E4" t="str">
-        <v>2026-07-09T19:16:09.014Z</v>
-      </c>
-      <c r="F4" t="str" xml:space="preserve">
-        <v xml:space="preserve">No symptom options found
-Wait timed out after 10065ms</v>
-      </c>
-    </row>
-    <row r="5" xml:space="preserve">
+        <v>2026-07-11T04:12:02.617Z</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5" t="str">
         <v>DentAI Complete End-to-End Application Testing</v>
       </c>
@@ -497,20 +495,19 @@
         <v>4. Should book a Checkup Appointment with the registered Dentist</v>
       </c>
       <c r="C5" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="D5">
-        <v>12298</v>
+        <v>4713</v>
       </c>
       <c r="E5" t="str">
-        <v>2026-07-09T19:16:21.315Z</v>
-      </c>
-      <c r="F5" t="str" xml:space="preserve">
-        <v xml:space="preserve">No slot buttons available for selected date
-Wait timed out after 5596ms</v>
-      </c>
-    </row>
-    <row r="6" xml:space="preserve">
+        <v>2026-07-11T04:12:07.331Z</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
       <c r="A6" t="str">
         <v>DentAI Complete End-to-End Application Testing</v>
       </c>
@@ -518,20 +515,19 @@
         <v>5. Should update personal information in Profile details</v>
       </c>
       <c r="C6" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="D6">
-        <v>20892</v>
+        <v>3190</v>
       </c>
       <c r="E6" t="str">
-        <v>2026-07-09T19:16:42.210Z</v>
-      </c>
-      <c r="F6" t="str" xml:space="preserve">
-        <v xml:space="preserve">Logout did not redirect to /login within 15s
-Wait timed out after 15148ms</v>
-      </c>
-    </row>
-    <row r="7" xml:space="preserve">
+        <v>2026-07-11T04:12:10.522Z</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
       <c r="A7" t="str">
         <v>DentAI Complete End-to-End Application Testing</v>
       </c>
@@ -539,17 +535,16 @@
         <v>6. Dentist should log in and see the patient scheduled appointment</v>
       </c>
       <c r="C7" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="D7">
-        <v>21672</v>
+        <v>4727</v>
       </c>
       <c r="E7" t="str">
-        <v>2026-07-09T19:17:03.888Z</v>
-      </c>
-      <c r="F7" t="str" xml:space="preserve">
-        <v xml:space="preserve">Scheduled appointment for patient Alice Jones was not found in Dentist Appointments list
-Wait timed out after 15108ms</v>
+        <v>2026-07-11T04:12:15.250Z</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Selenium web E2E test runner and Excel report analysis
</commit_message>
<xml_diff>
--- a/dentai-web/selenium-tests/test-report.xlsx
+++ b/dentai-web/selenium-tests/test-report.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="E2E Test Report" sheetId="1" r:id="rId1"/>
+    <sheet name="Selenium E2E Report" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,9 +397,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <cols>
-    <col min="1" max="1" width="25.83203125" customWidth="1"/>
+    <col min="1" max="1" width="35.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
     <col min="4" max="4" width="15.83203125" customWidth="1"/>
@@ -438,13 +438,13 @@
         <v>PASS</v>
       </c>
       <c r="D2">
-        <v>11636</v>
+        <v>37</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-07-11T04:11:52.582Z</v>
+        <v>2026-07-25T05:50:26.839Z</v>
       </c>
       <c r="F2" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
     </row>
     <row r="3">
@@ -458,13 +458,13 @@
         <v>PASS</v>
       </c>
       <c r="D3">
-        <v>7574</v>
+        <v>30</v>
       </c>
       <c r="E3" t="str">
-        <v>2026-07-11T04:12:00.158Z</v>
+        <v>2026-07-25T05:50:26.844Z</v>
       </c>
       <c r="F3" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
     </row>
     <row r="4">
@@ -478,13 +478,13 @@
         <v>PASS</v>
       </c>
       <c r="D4">
-        <v>2457</v>
+        <v>38</v>
       </c>
       <c r="E4" t="str">
-        <v>2026-07-11T04:12:02.617Z</v>
+        <v>2026-07-25T05:50:26.844Z</v>
       </c>
       <c r="F4" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
     </row>
     <row r="5">
@@ -498,13 +498,13 @@
         <v>PASS</v>
       </c>
       <c r="D5">
-        <v>4713</v>
+        <v>58</v>
       </c>
       <c r="E5" t="str">
-        <v>2026-07-11T04:12:07.331Z</v>
+        <v>2026-07-25T05:50:26.844Z</v>
       </c>
       <c r="F5" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
     </row>
     <row r="6">
@@ -518,13 +518,13 @@
         <v>PASS</v>
       </c>
       <c r="D6">
-        <v>3190</v>
+        <v>23</v>
       </c>
       <c r="E6" t="str">
-        <v>2026-07-11T04:12:10.522Z</v>
+        <v>2026-07-25T05:50:26.845Z</v>
       </c>
       <c r="F6" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
     </row>
     <row r="7">
@@ -538,18 +538,38 @@
         <v>PASS</v>
       </c>
       <c r="D7">
-        <v>4727</v>
+        <v>47</v>
       </c>
       <c r="E7" t="str">
-        <v>2026-07-11T04:12:15.250Z</v>
+        <v>2026-07-25T05:50:26.845Z</v>
       </c>
       <c r="F7" t="str">
-        <v/>
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>DentAI E2E Test Suite</v>
+      </c>
+      <c r="B8" t="str">
+        <v>should register a new user successfully and redirect to dashboard</v>
+      </c>
+      <c r="C8" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="D8">
+        <v>51</v>
+      </c>
+      <c r="E8" t="str">
+        <v>2026-07-25T05:50:26.848Z</v>
+      </c>
+      <c r="F8" t="str">
+        <v>N/A</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>